<commit_message>
feat: add tax and labor rules
</commit_message>
<xml_diff>
--- a/data/processed/ontology/enterprise/predicate_lexicon.xlsx
+++ b/data/processed/ontology/enterprise/predicate_lexicon.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N75"/>
+  <dimension ref="A1:N70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2959,27 +2959,27 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>PRED_CAP_LAI_GIAY_CHUNG_NHAN_DANG_KY_DOANH_NGHIEP_VA_CAP_</t>
+          <t>PRED_XEM_XET_VA_CAP_GIAY_CHUNG_NHAN_DANG_KY_DOANH_NGHIEP</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>cấp lại Giấy chứng nhận đăng ký doanh nghiệp và cập nhật tình trạng pháp lý của công ty trên Cơ sở dữ liệu quốc gia về đăng ký doanh nghiệp.</t>
+          <t>xem xét và cấp Giấy chứng nhận đăng ký doanh nghiệp</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>cấp lại Giấy chứng nhận đăng ký doanh nghiệp và cập nhật tình trạng pháp lý của công ty trên Cơ sở dữ liệu quốc gia về đăng ký doanh nghiệp. | cấp lại Giấy chứng nhận đăng ký doanh nghiệp và cập nhật tình trạng pháp lý của công ty trên Cơ sở dữ liệu quốc gia về đăng ký doanh nghiệp. với cơ quan đăng ký kinh doanh</t>
+          <t>xem xét và cấp Giấy chứng nhận đăng ký doanh nghiệp | xem xét và cấp Giấy chứng nhận đăng ký doanh nghiệp với cơ quan đăng ký kinh doanh</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>khac</t>
+          <t>tham_dinh_ho_so</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>cap_lai_giay_chung_nhan_dang_ky_doanh_nghiep_va_cap_nhat_tinh_trang_phap_ly_cua_cong_ty_tren_co_so_du_lieu_quoc_gia_ve_dang_ky_doanh_nghiep</t>
+          <t>xem_xet_va_cap_giay_chung_nhan_dang_ky_doanh_nghiep</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -3024,39 +3024,39 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>map_khi_thay_cum_cap_lai_giay_chung_nhan_dang_ky_doanh_nghiep_va_cap_nhat_tinh_trang_phap_ly_cua_cong_ty_tren_co_so_du_lieu_quoc_gia_ve_dang_ky_doanh_nghiep;thuong_di_kem_thoi_han</t>
+          <t>map_khi_thay_cum_xem_xet_va_cap_giay_chung_nhan_dang_ky_doanh_nghiep;thuong_di_kem_thoi_han</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>PRED_XEM_XET_VA_CAP_GIAY_CHUNG_NHAN_DANG_KY_DOANH_NGHIEP</t>
+          <t>PRED_NEU_CO_DU_DIEU_KIEN_QUY_DINH_TAI_KHOAN_1_DIEU_NAY_VA</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>xem xét và cấp Giấy chứng nhận đăng ký doanh nghiệp</t>
+          <t>nếu có đủ điều kiện quy định tại khoản 1 Điều này và cập nhật tình trạng pháp lý của doanh nghiệp trên Cơ sở dữ liệu quốc gia về đăng ký doanh nghiệp.</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>xem xét và cấp Giấy chứng nhận đăng ký doanh nghiệp | xem xét và cấp Giấy chứng nhận đăng ký doanh nghiệp với cơ quan đăng ký kinh doanh</t>
+          <t>nếu có đủ điều kiện quy định tại khoản 1 Điều này và cập nhật tình trạng pháp lý của doanh nghiệp trên Cơ sở dữ liệu quốc gia về đăng ký doanh nghiệp. | nếu có đủ điều kiện quy định tại khoản 1 Điều này và cập nhật tình trạng pháp lý của doanh nghiệp trên Cơ sở dữ liệu quốc gia về đăng ký doanh nghiệp. với cơ quan đăng ký kinh doanh</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>tham_dinh_ho_so</t>
+          <t>dieu_kien_ap_dung</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>xem_xet_va_cap_giay_chung_nhan_dang_ky_doanh_nghiep</t>
+          <t>neu_co_du_dieu_kien_quy_dinh_tai_khoan_1_dieu_nay_va_cap_nhat_tinh_trang_phap_ly_cua_doanh_nghiep_tren_co_so_du_lieu_quoc_gia_ve_dang_ky_doanh_nghiep</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>hanh_dong_co_quan</t>
+          <t>dieu_kien</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -3096,7 +3096,7 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>map_khi_thay_cum_xem_xet_va_cap_giay_chung_nhan_dang_ky_doanh_nghiep;thuong_di_kem_thoi_han</t>
+          <t>map_cho_ve_dieu_kien_ap_dung;uu_tien_giu_nguyen_ngu_canh</t>
         </is>
       </c>
     </row>
@@ -3108,12 +3108,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>nếu có đủ điều kiện quy định tại khoản 1 Điều này và cập nhật tình trạng pháp lý của doanh nghiệp trên Cơ sở dữ liệu quốc gia về đăng ký doanh nghiệp.</t>
+          <t>nếu có đủ điều kiện quy định tại khoản 1 Điều này và cập nhật tình trạng pháp lý của doanh nghiệp trên Cơ sở dữ liệu quốc gia về</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>nếu có đủ điều kiện quy định tại khoản 1 Điều này và cập nhật tình trạng pháp lý của doanh nghiệp trên Cơ sở dữ liệu quốc gia về đăng ký doanh nghiệp. | nếu có đủ điều kiện quy định tại khoản 1 Điều này và cập nhật tình trạng pháp lý của doanh nghiệp trên Cơ sở dữ liệu quốc gia về đăng ký doanh nghiệp. với cơ quan đăng ký kinh doanh</t>
+          <t>nếu có đủ điều kiện quy định tại khoản 1 Điều này và cập nhật tình trạng pháp lý của doanh nghiệp trên Cơ sở dữ liệu quốc gia về | nếu có đủ điều kiện quy định tại khoản 1 Điều này và cập nhật tình trạng pháp lý của doanh nghiệp trên Cơ sở dữ liệu quốc gia về với cơ quan đăng ký kinh doanh</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -3123,7 +3123,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>neu_co_du_dieu_kien_quy_dinh_tai_khoan_1_dieu_nay_va_cap_nhat_tinh_trang_phap_ly_cua_doanh_nghiep_tren_co_so_du_lieu_quoc_gia_ve_dang_ky_doanh_nghiep</t>
+          <t>neu_co_du_dieu_kien_quy_dinh_tai_khoan_1_dieu_nay_va_cap_nhat_tinh_trang_phap_ly_cua_doanh_nghiep_tren_co_so_du_lieu_quoc_gia_ve</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -3175,32 +3175,32 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>PRED_NEU_CO_DU_DIEU_KIEN_QUY_DINH_TAI_KHOAN_1_DIEU_NAY_VA</t>
+          <t>PRED_GIAY_CHUNG_NHAN_DANG_KY_DOANH_NGHIEP</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>nếu có đủ điều kiện quy định tại khoản 1 Điều này và cập nhật tình trạng pháp lý của doanh nghiệp trên Cơ sở dữ liệu quốc gia về</t>
+          <t>Giấy chứng nhận đăng ký doanh nghiệp</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>nếu có đủ điều kiện quy định tại khoản 1 Điều này và cập nhật tình trạng pháp lý của doanh nghiệp trên Cơ sở dữ liệu quốc gia về | nếu có đủ điều kiện quy định tại khoản 1 Điều này và cập nhật tình trạng pháp lý của doanh nghiệp trên Cơ sở dữ liệu quốc gia về với cơ quan đăng ký kinh doanh</t>
+          <t>Giấy chứng nhận đăng ký doanh nghiệp | Giấy chứng nhận đăng ký doanh nghiệp với cơ quan đăng ký kinh doanh</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>dieu_kien_ap_dung</t>
+          <t>dang_ky</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>neu_co_du_dieu_kien_quy_dinh_tai_khoan_1_dieu_nay_va_cap_nhat_tinh_trang_phap_ly_cua_doanh_nghiep_tren_co_so_du_lieu_quoc_gia_ve</t>
+          <t>giay_chung_nhan_dang_ky_doanh_nghiep</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>dieu_kien</t>
+          <t>dang_ky</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -3235,61 +3235,61 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>co</t>
+          <t>khong</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>map_cho_ve_dieu_kien_ap_dung;uu_tien_giu_nguyen_ngu_canh</t>
+          <t>map_khi_thay_cum_giay_chung_nhan_dang_ky_doanh_nghiep;uu_tien_cho_hanh_vi_dang_ky_noi_dung_phap_ly;thuong_di_kem_thoi_han</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>PRED_GIAY_CHUNG_NHAN_DANG_KY_DOANH_NGHIEP</t>
+          <t>PRED_THONG_BAO_BANG_VAN_BAN</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Giấy chứng nhận đăng ký doanh nghiệp</t>
+          <t>thông báo bằng văn bản cho Cơ quan đăng ký kinh doanh</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Giấy chứng nhận đăng ký doanh nghiệp | Giấy chứng nhận đăng ký doanh nghiệp với cơ quan đăng ký kinh doanh</t>
+          <t>thông báo bằng văn bản cho Cơ quan đăng ký kinh doanh | thông báo bằng văn bản cho Cơ quan đăng ký kinh doanh với cơ quan đăng ký kinh doanh</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>dang_ky</t>
+          <t>thong_bao</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>giay_chung_nhan_dang_ky_doanh_nghiep</t>
+          <t>thong_bao_bang_van_ban</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>dang_ky</t>
+          <t>thong_bao</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
+          <t>doanh nghiệp</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>chậm nhất là 03 ngày làm việc trước ngày tạm ngừng kinh doanh hoặc tiếp tục kinh doanh trước thời hạn đã thông báo</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
           <t>cơ quan đăng ký kinh doanh</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>Giấy chứng nhận đăng ký doanh nghiệp</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>cơ quan đăng ký kinh doanh</t>
-        </is>
-      </c>
       <c r="J42" t="inlineStr">
         <is>
           <t>co</t>
@@ -3312,49 +3312,49 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>map_khi_thay_cum_giay_chung_nhan_dang_ky_doanh_nghiep;uu_tien_cho_hanh_vi_dang_ky_noi_dung_phap_ly;thuong_di_kem_thoi_han</t>
+          <t>map_khi_thay_cum_thong_bao_bang_van_ban;khong_dong_nhat_voi_cong_bo;thuong_di_kem_thoi_han</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>PRED_THONG_BAO_BANG_VAN_BAN</t>
+          <t>PRED_GUI_HO_SO</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>thông báo bằng văn bản cho Cơ quan đăng ký kinh doanh</t>
+          <t>gửi hồ sơ giải thể doanh nghiệp cho Cơ quan đăng ký kinh doanh</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>thông báo bằng văn bản cho Cơ quan đăng ký kinh doanh | thông báo bằng văn bản cho Cơ quan đăng ký kinh doanh với cơ quan đăng ký kinh doanh</t>
+          <t>gửi hồ sơ giải thể doanh nghiệp cho Cơ quan đăng ký kinh doanh | gửi hồ sơ giải thể doanh nghiệp cho Cơ quan đăng ký kinh doanh với cơ quan đăng ký kinh doanh</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>thong_bao</t>
+          <t>nop_ho_so</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>thong_bao_bang_van_ban</t>
+          <t>gui_ho_so</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>thong_bao</t>
+          <t>nop_ho_so</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>doanh nghiệp</t>
+          <t>cơ quan đăng ký kinh doanh</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>chậm nhất là 03 ngày làm việc trước ngày tạm ngừng kinh doanh hoặc tiếp tục kinh doanh trước thời hạn đã thông báo</t>
+          <t>thời hạn</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3384,59 +3384,55 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>map_khi_thay_cum_thong_bao_bang_van_ban;khong_dong_nhat_voi_cong_bo;thuong_di_kem_thoi_han</t>
+          <t>map_khi_thay_cum_gui_ho_so;thuong_di_kem_thoi_han</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>PRED_GUI_HO_SO</t>
+          <t>PRED_THU_HOI</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>gửi hồ sơ giải thể doanh nghiệp cho Cơ quan đăng ký kinh doanh</t>
+          <t>thu hồi Giấy chứng nhận đăng ký doanh nghiệp trong</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>gửi hồ sơ giải thể doanh nghiệp cho Cơ quan đăng ký kinh doanh | gửi hồ sơ giải thể doanh nghiệp cho Cơ quan đăng ký kinh doanh với cơ quan đăng ký kinh doanh</t>
+          <t>thu hồi Giấy chứng nhận đăng ký doanh nghiệp trong</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>nop_ho_so</t>
+          <t>thu_hoi</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>gui_ho_so</t>
+          <t>thu_hoi</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>nop_ho_so</t>
+          <t>thu_hoi</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>cơ quan đăng ký kinh doanh</t>
+          <t>doanh nghiệp</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>thời hạn</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>cơ quan đăng ký kinh doanh</t>
-        </is>
-      </c>
+          <t>Giấy chứng nhận đăng ký doanh nghiệp</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr">
         <is>
-          <t>co</t>
+          <t>khong</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3456,39 +3452,39 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>map_khi_thay_cum_gui_ho_so;thuong_di_kem_thoi_han</t>
+          <t>map_khi_thay_cum_thu_hoi</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>PRED_THU_HOI</t>
+          <t>PRED_CAP_DANG_KY_CO_TRACH_NHIEM_TICH_HOP</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>thu hồi Giấy chứng nhận đăng ký doanh nghiệp trong</t>
+          <t>cấp đăng ký có trách nhiệm tích hợp</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>thu hồi Giấy chứng nhận đăng ký doanh nghiệp trong</t>
+          <t>cấp đăng ký có trách nhiệm tích hợp | cấp đăng ký có trách nhiệm tích hợp với cơ quan đăng ký kinh doanh</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>thu_hoi</t>
+          <t>cap_giay</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>thu_hoi</t>
+          <t>cap_dang_ky_co_trach_nhiem_tich_hop</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>thu_hoi</t>
+          <t>cap_giay</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -3496,12 +3492,12 @@
           <t>doanh nghiệp</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>Giấy chứng nhận đăng ký doanh nghiệp</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>cơ quan đăng ký kinh doanh</t>
+        </is>
+      </c>
       <c r="J45" t="inlineStr">
         <is>
           <t>khong</t>
@@ -3524,39 +3520,39 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>map_khi_thay_cum_thu_hoi</t>
+          <t>map_khi_thay_cum_cap_dang_ky_co_trach_nhiem_tich_hop</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>PRED_CAP_DANG_KY_CO_TRACH_NHIEM_TICH_HOP</t>
+          <t>PRED_VA_CAC_CO_QUAN_KHAC_GAY_PHIEN_HA</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>cấp đăng ký có trách nhiệm tích hợp</t>
+          <t>Cơ quan đăng ký kinh doanh và các cơ quan khác gây phiền hà</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>cấp đăng ký có trách nhiệm tích hợp | cấp đăng ký có trách nhiệm tích hợp với cơ quan đăng ký kinh doanh</t>
+          <t>Cơ quan đăng ký kinh doanh và các cơ quan khác gây phiền hà | Cơ quan đăng ký kinh doanh và các cơ quan khác gây phiền hà với cơ quan đăng ký kinh doanh</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>cap_giay</t>
+          <t>dang_ky</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>cap_dang_ky_co_trach_nhiem_tich_hop</t>
+          <t>va_cac_co_quan_khac_gay_phien_ha</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>cap_giay</t>
+          <t>dang_ky</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -3564,7 +3560,11 @@
           <t>doanh nghiệp</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr"/>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>tổ chức</t>
+        </is>
+      </c>
       <c r="I46" t="inlineStr">
         <is>
           <t>cơ quan đăng ký kinh doanh</t>
@@ -3592,24 +3592,24 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>map_khi_thay_cum_cap_dang_ky_co_trach_nhiem_tich_hop</t>
+          <t>map_khi_thay_cum_va_cac_co_quan_khac_gay_phien_ha;uu_tien_cho_hanh_vi_dang_ky_noi_dung_phap_ly</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>PRED_VIEC_BO_SUNG_THONG_TIN_VE_CHU_SO_HUU_HUONG_LOI_CUA_D</t>
+          <t>PRED_CAP_LAI_CHO_TO_CHUC</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>việc bổ sung thông tin về chủ sở hữu hưởng lợi của doanh nghiệp (</t>
+          <t>cấp lại cho tổ chức</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>việc bổ sung thông tin về chủ sở hữu hưởng lợi của doanh nghiệp (</t>
+          <t>cấp lại cho tổ chức | cấp lại cho tổ chức với cơ quan đăng ký kinh doanh</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -3619,12 +3619,12 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>viec_bo_sung_thong_tin_ve_chu_so_huu_huong_loi_cua_doanh_nghiep</t>
+          <t>cap_lai_cho_to_chuc</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>chu_so_huu_huong_loi</t>
+          <t>hanh_dong_co_quan</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -3632,12 +3632,12 @@
           <t>doanh nghiệp</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>nội dung đăng ký doanh nghiệp</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>cơ quan đăng ký kinh doanh</t>
+        </is>
+      </c>
       <c r="J47" t="inlineStr">
         <is>
           <t>khong</t>
@@ -3650,7 +3650,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>co</t>
+          <t>khong</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
@@ -3660,39 +3660,39 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>map_khi_thay_cum_viec_bo_sung_thong_tin_ve_chu_so_huu_huong_loi_cua_doanh_nghiep;co_ngoai_le_can_xu_ly_rieng</t>
+          <t>map_khi_thay_cum_cap_lai_cho_to_chuc</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>PRED_VA_CAC_CO_QUAN_KHAC_GAY_PHIEN_HA</t>
+          <t>PRED_KEM_THEO_TAI_LIEU_BANG_TIENG_NUOC_NGOAI</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Cơ quan đăng ký kinh doanh và các cơ quan khác gây phiền hà</t>
+          <t>kèm theo tài liệu bằng tiếng nước ngoài.</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Cơ quan đăng ký kinh doanh và các cơ quan khác gây phiền hà | Cơ quan đăng ký kinh doanh và các cơ quan khác gây phiền hà với cơ quan đăng ký kinh doanh</t>
+          <t>kèm theo tài liệu bằng tiếng nước ngoài.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>dang_ky</t>
+          <t>nop_ho_so</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>va_cac_co_quan_khac_gay_phien_ha</t>
+          <t>kem_theo_tai_lieu_bang_tieng_nuoc_ngoai</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>dang_ky</t>
+          <t>nop_ho_so</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -3702,14 +3702,10 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>tổ chức</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>cơ quan đăng ký kinh doanh</t>
-        </is>
-      </c>
+          <t>hồ sơ đăng ký doanh nghiệp</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr">
         <is>
           <t>khong</t>
@@ -3717,7 +3713,7 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>khong</t>
+          <t>co</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
@@ -3732,39 +3728,39 @@
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>map_khi_thay_cum_va_cac_co_quan_khac_gay_phien_ha;uu_tien_cho_hanh_vi_dang_ky_noi_dung_phap_ly</t>
+          <t>map_khi_noi_dung_la_thanh_phan_ho_so_hoac_giay_to_kem_theo</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>PRED_CAP_LAI_CHO_TO_CHUC</t>
+          <t>PRED_KEM_THEO_HO_SO</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>cấp lại cho tổ chức</t>
+          <t>kèm theo hồ sơ</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>cấp lại cho tổ chức | cấp lại cho tổ chức với cơ quan đăng ký kinh doanh</t>
+          <t>kèm theo hồ sơ</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>khac</t>
+          <t>nop_ho_so</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>cap_lai_cho_to_chuc</t>
+          <t>kem_theo_ho_so</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>hanh_dong_co_quan</t>
+          <t>nop_ho_so</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -3772,12 +3768,12 @@
           <t>doanh nghiệp</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>cơ quan đăng ký kinh doanh</t>
-        </is>
-      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>hồ sơ đăng ký doanh nghiệp</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr">
         <is>
           <t>khong</t>
@@ -3785,7 +3781,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>khong</t>
+          <t>co</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
@@ -3800,24 +3796,24 @@
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>map_khi_thay_cum_cap_lai_cho_to_chuc</t>
+          <t>map_khi_thay_cum_kem_theo_ho_so;thuong_di_kem_thanh_phan_ho_so</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>PRED_KEM_THEO_TAI_LIEU_BANG_TIENG_NUOC_NGOAI</t>
+          <t>PRED_VAN_BAN_UY_QUYEN</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>kèm theo tài liệu bằng tiếng nước ngoài.</t>
+          <t>Văn bản ủy quyền; Giấy đề nghị đăng ký doanh nghiệp</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>kèm theo tài liệu bằng tiếng nước ngoài.</t>
+          <t>Văn bản ủy quyền; Giấy đề nghị đăng ký doanh nghiệp</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -3827,7 +3823,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>kem_theo_tai_lieu_bang_tieng_nuoc_ngoai</t>
+          <t>van_ban_uy_quyen</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -3875,53 +3871,57 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>PRED_KEM_THEO_HO_SO</t>
+          <t>PRED_CAP_DANG_KY_DOANH_NGHIEP</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>kèm theo hồ sơ</t>
+          <t>cấp đăng ký doanh nghiệp theo quy trình dự phòng</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>kèm theo hồ sơ</t>
+          <t>cấp đăng ký doanh nghiệp theo quy trình dự phòng | cấp đăng ký doanh nghiệp theo quy trình dự phòng với cơ quan đăng ký kinh doanh</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>nop_ho_so</t>
+          <t>cap_giay</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>kem_theo_ho_so</t>
+          <t>cap_dang_ky_doanh_nghiep</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>nop_ho_so</t>
+          <t>cap_giay</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>doanh nghiệp</t>
+          <t>cơ quan đăng ký kinh doanh</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>hồ sơ đăng ký doanh nghiệp</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr"/>
+          <t>dang_ky_doanh_nghiep</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>cơ quan đăng ký kinh doanh</t>
+        </is>
+      </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>khong</t>
+          <t>co</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>co</t>
+          <t>khong</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
@@ -3931,65 +3931,61 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>khong</t>
+          <t>co</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>map_khi_thay_cum_kem_theo_ho_so;thuong_di_kem_thanh_phan_ho_so</t>
+          <t>map_khi_thay_cum_cap_dang_ky_doanh_nghiep;thuong_di_kem_thoi_han</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>PRED_VAN_BAN_UY_QUYEN</t>
+          <t>PRED_DANG_KY_DOANH_NGHIEP</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Văn bản ủy quyền; Giấy đề nghị đăng ký doanh nghiệp</t>
+          <t>đăng ký thay đổi tên. Doanh nghiệp có tên vi phạm phải đăng ký thay đổi tên doanh nghiệp</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Văn bản ủy quyền; Giấy đề nghị đăng ký doanh nghiệp</t>
+          <t>đăng ký thay đổi tên. Doanh nghiệp có tên vi phạm phải đăng ký thay đổi tên doanh nghiệp | đăng ký thay đổi tên. Doanh nghiệp có tên vi phạm phải đăng ký thay đổi tên doanh nghiệp với cơ quan đăng ký kinh doanh</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>nop_ho_so</t>
+          <t>dang_ky</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>van_ban_uy_quyen</t>
+          <t>dang_ky_doanh_nghiep</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>nop_ho_so</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>doanh nghiệp</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>hồ sơ đăng ký doanh nghiệp</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr"/>
+          <t>ten_doanh_nghiep</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>cơ quan đăng ký kinh doanh</t>
+        </is>
+      </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>khong</t>
+          <t>co</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>co</t>
+          <t>khong</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
@@ -4004,59 +4000,55 @@
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>map_khi_noi_dung_la_thanh_phan_ho_so_hoac_giay_to_kem_theo</t>
+          <t>map_khi_thay_cum_dang_ky_doanh_nghiep;thuong_di_kem_thoi_han</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>PRED_CAP_DANG_KY_DOANH_NGHIEP</t>
+          <t>PRED_NEU_CONG_TY</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>cấp đăng ký doanh nghiệp theo quy trình dự phòng</t>
+          <t>nếu công ty</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>cấp đăng ký doanh nghiệp theo quy trình dự phòng | cấp đăng ký doanh nghiệp theo quy trình dự phòng với cơ quan đăng ký kinh doanh</t>
+          <t>nếu công ty</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>cap_giay</t>
+          <t>dieu_kien_ap_dung</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>cap_dang_ky_doanh_nghiep</t>
+          <t>neu_cong_ty</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>cap_giay</t>
+          <t>dieu_kien</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>cơ quan đăng ký kinh doanh</t>
+          <t>công ty cổ phần</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>dang_ky_doanh_nghiep</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>cơ quan đăng ký kinh doanh</t>
-        </is>
-      </c>
+          <t>cổ đông sáng lập</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr">
         <is>
-          <t>co</t>
+          <t>khong</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -4071,29 +4063,29 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>co</t>
+          <t>khong</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>map_khi_thay_cum_cap_dang_ky_doanh_nghiep;thuong_di_kem_thoi_han</t>
+          <t>map_cho_ve_dieu_kien_ap_dung;uu_tien_giu_nguyen_ngu_canh</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>PRED_TIEP_TUC_SU_DUNG_TEN_DOANH_NGHIEP_DA_DANG_KY_VA_KHON</t>
+          <t>PRED_LAP_DIA_DIEM_KINH_DOANH_DEN_CO_QUAN</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>tiếp tục sử dụng tên doanh nghiệp đã đăng ký và không bắt buộc phải đăng ký đổi tên doanh nghiệp trong</t>
+          <t>lập địa điểm kinh doanh đến Cơ quan</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>tiếp tục sử dụng tên doanh nghiệp đã đăng ký và không bắt buộc phải đăng ký đổi tên doanh nghiệp trong</t>
+          <t>lập địa điểm kinh doanh đến Cơ quan | lập địa điểm kinh doanh đến Cơ quan với cơ quan đăng ký kinh doanh cấp tỉnh</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -4103,12 +4095,12 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>tiep_tuc_su_dung_ten_doanh_nghiep_da_dang_ky_va_khong_bat_buoc_phai_dang_ky_doi_ten_doanh_nghiep_trong</t>
+          <t>lap_dia_diem_kinh_doanh_den_co_quan</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>ten_doanh_nghiep</t>
+          <t>chi_nhanh_van_phong_dai_dien</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -4118,13 +4110,17 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>trường hợp có tên trùng</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr"/>
+          <t>đăng ký kinh doanh cấp tỉnh nơi đặt địa điểm kinh doanh</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>cơ quan đăng ký kinh doanh cấp tỉnh</t>
+        </is>
+      </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>khong</t>
+          <t>co</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -4139,51 +4135,59 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>khong</t>
+          <t>co</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>map_khi_thay_cum_tiep_tuc_su_dung_ten_doanh_nghiep_da_dang_ky_va_khong_bat_buoc_phai_dang_ky_doi_ten_doanh_nghiep_trong</t>
+          <t>map_khi_thay_cum_lap_dia_diem_kinh_doanh_den_co_quan;thuong_di_kem_thoi_han</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>PRED_DANG_KY_DOANH_NGHIEP</t>
+          <t>PRED_CAP_GIAY_CHUNG_NHAN_DANG_KY_HOAT_DONG_CHI_NHANH</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>đăng ký thay đổi tên. Doanh nghiệp có tên vi phạm phải đăng ký thay đổi tên doanh nghiệp</t>
+          <t>cấp tỉnh cấp Giấy chứng nhận đăng ký hoạt động chi nhánh</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>đăng ký thay đổi tên. Doanh nghiệp có tên vi phạm phải đăng ký thay đổi tên doanh nghiệp | đăng ký thay đổi tên. Doanh nghiệp có tên vi phạm phải đăng ký thay đổi tên doanh nghiệp với cơ quan đăng ký kinh doanh</t>
+          <t>cấp tỉnh cấp Giấy chứng nhận đăng ký hoạt động chi nhánh | cấp tỉnh cấp Giấy chứng nhận đăng ký hoạt động chi nhánh với cơ quan đăng ký kinh doanh cấp tỉnh</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>dang_ky</t>
+          <t>cap_giay</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>dang_ky_doanh_nghiep</t>
+          <t>cap_giay_chung_nhan_dang_ky_hoat_dong_chi_nhanh</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>ten_doanh_nghiep</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
+          <t>cap_giay</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>cơ quan đăng ký kinh doanh</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>chi_nhanh</t>
+        </is>
+      </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>cơ quan đăng ký kinh doanh</t>
+          <t>cơ quan đăng ký kinh doanh cấp tỉnh</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -4203,54 +4207,54 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>khong</t>
+          <t>co</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>map_khi_thay_cum_dang_ky_doanh_nghiep;thuong_di_kem_thoi_han</t>
+          <t>map_khi_thay_cum_cap_giay_chung_nhan_dang_ky_hoat_dong_chi_nhanh;thuong_di_kem_thoi_han</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>PRED_NEU_CONG_TY</t>
+          <t>PRED_TIEP_NHAN_DE_NHAP_THONG_TIN_VAO_HE_THONG_THONG_TIN_Q</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>nếu công ty</t>
+          <t>tiếp nhận để nhập thông tin vào Hệ thống thông tin quốc gia về đăng ký doanh nghiệp</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>nếu công ty</t>
+          <t>tiếp nhận để nhập thông tin vào Hệ thống thông tin quốc gia về đăng ký doanh nghiệp</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>dieu_kien_ap_dung</t>
+          <t>tiep_nhan_ho_so</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>neu_cong_ty</t>
+          <t>tiep_nhan_de_nhap_thong_tin_vao_he_thong_thong_tin_quoc_gia_ve_dang_ky_doanh_nghiep</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>dieu_kien</t>
+          <t>hanh_dong_co_quan</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>công ty cổ phần</t>
+          <t>doanh nghiệp</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>cổ đông sáng lập</t>
+          <t>Hồ sơ đăng ký doanh nghiệp</t>
         </is>
       </c>
       <c r="I56" t="inlineStr"/>
@@ -4276,49 +4280,49 @@
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>map_cho_ve_dieu_kien_ap_dung;uu_tien_giu_nguyen_ngu_canh</t>
+          <t>map_khi_thay_cum_tiep_nhan_de_nhap_thong_tin_vao_he_thong_thong_tin_quoc_gia_ve_dang_ky_doanh_nghiep</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>PRED_LAP_DIA_DIEM_KINH_DOANH_DEN_CO_QUAN</t>
+          <t>PRED_TRAO_GIAY_TIEP_NHAN_HO_SO_VA_HEN_TRA_KET_QUA_CHO_NGU</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>lập địa điểm kinh doanh đến Cơ quan</t>
+          <t>cấp tỉnh trao giấy tiếp nhận hồ sơ và hẹn trả kết quả cho người nộp hồ sơ.</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>lập địa điểm kinh doanh đến Cơ quan | lập địa điểm kinh doanh đến Cơ quan với cơ quan đăng ký kinh doanh cấp tỉnh</t>
+          <t>cấp tỉnh trao giấy tiếp nhận hồ sơ và hẹn trả kết quả cho người nộp hồ sơ. | cấp tỉnh trao giấy tiếp nhận hồ sơ và hẹn trả kết quả cho người nộp hồ sơ. với cơ quan đăng ký kinh doanh cấp tỉnh</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>khac</t>
+          <t>nop_ho_so</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>lap_dia_diem_kinh_doanh_den_co_quan</t>
+          <t>trao_giay_tiep_nhan_ho_so_va_hen_tra_ket_qua_cho_nguoi_nop_ho_so</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>chi_nhanh_van_phong_dai_dien</t>
+          <t>nop_ho_so</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>doanh nghiệp</t>
+          <t>cơ quan đăng ký kinh doanh</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>đăng ký kinh doanh cấp tỉnh nơi đặt địa điểm kinh doanh</t>
+          <t>hồ sơ đăng ký doanh nghiệp</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -4328,7 +4332,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>co</t>
+          <t>khong</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -4343,54 +4347,54 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>co</t>
+          <t>khong</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>map_khi_thay_cum_lap_dia_diem_kinh_doanh_den_co_quan;thuong_di_kem_thoi_han</t>
+          <t>map_khi_thay_cum_trao_giay_tiep_nhan_ho_so_va_hen_tra_ket_qua_cho_nguoi_nop_ho_so</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>PRED_CAP_GIAY_CHUNG_NHAN_DANG_KY_HOAT_DONG_CHI_NHANH</t>
+          <t>PRED_DUNG_THUC_HIEN_THU_TUC_DANG_KY_DOANH_NGHIEP</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>cấp tỉnh cấp Giấy chứng nhận đăng ký hoạt động chi nhánh</t>
+          <t>dừng thực hiện thủ tục đăng ký doanh nghiệp</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>cấp tỉnh cấp Giấy chứng nhận đăng ký hoạt động chi nhánh | cấp tỉnh cấp Giấy chứng nhận đăng ký hoạt động chi nhánh với cơ quan đăng ký kinh doanh cấp tỉnh</t>
+          <t>dừng thực hiện thủ tục đăng ký doanh nghiệp | dừng thực hiện thủ tục đăng ký doanh nghiệp với cơ quan đăng ký kinh doanh cấp tỉnh</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>cap_giay</t>
+          <t>dang_ky</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>cap_giay_chung_nhan_dang_ky_hoat_dong_chi_nhanh</t>
+          <t>dung_thuc_hien_thu_tuc_dang_ky_doanh_nghiep</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>cap_giay</t>
+          <t>dang_ky</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>cơ quan đăng ký kinh doanh</t>
+          <t>người thành lập doanh nghiệp</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>chi_nhanh</t>
+          <t>hồ sơ đăng ký doanh nghiệp</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -4415,60 +4419,64 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>co</t>
+          <t>khong</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
         <is>
-          <t>map_khi_thay_cum_cap_giay_chung_nhan_dang_ky_hoat_dong_chi_nhanh;thuong_di_kem_thoi_han</t>
+          <t>map_khi_thay_cum_dung_thuc_hien_thu_tuc_dang_ky_doanh_nghiep;uu_tien_cho_hanh_vi_dang_ky_noi_dung_phap_ly;thuong_di_kem_thoi_han</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>PRED_TIEP_NHAN_DE_NHAP_THONG_TIN_VAO_HE_THONG_THONG_TIN_Q</t>
+          <t>PRED_TRAO_GIAY_TIEP_NHAN_HO_SO_VA_HEN_TRA_KET_QUA</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>tiếp nhận để nhập thông tin vào Hệ thống thông tin quốc gia về đăng ký doanh nghiệp</t>
+          <t>cấp tỉnh trao giấy tiếp nhận hồ sơ và hẹn trả kết quả</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>tiếp nhận để nhập thông tin vào Hệ thống thông tin quốc gia về đăng ký doanh nghiệp</t>
+          <t>cấp tỉnh trao giấy tiếp nhận hồ sơ và hẹn trả kết quả | cấp tỉnh trao giấy tiếp nhận hồ sơ và hẹn trả kết quả với cơ quan đăng ký kinh doanh cấp tỉnh</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>tiep_nhan_ho_so</t>
+          <t>nop_ho_so</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>tiep_nhan_de_nhap_thong_tin_vao_he_thong_thong_tin_quoc_gia_ve_dang_ky_doanh_nghiep</t>
+          <t>trao_giay_tiep_nhan_ho_so_va_hen_tra_ket_qua</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>hanh_dong_co_quan</t>
+          <t>nop_ho_so</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>doanh nghiệp</t>
+          <t>cơ quan đăng ký kinh doanh</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Hồ sơ đăng ký doanh nghiệp</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr"/>
+          <t>Giấy chứng nhận đăng ký doanh nghiệp</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>cơ quan đăng ký kinh doanh cấp tỉnh</t>
+        </is>
+      </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>khong</t>
+          <t>co</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4488,24 +4496,24 @@
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>map_khi_thay_cum_tiep_nhan_de_nhap_thong_tin_vao_he_thong_thong_tin_quoc_gia_ve_dang_ky_doanh_nghiep</t>
+          <t>map_khi_thay_cum_trao_giay_tiep_nhan_ho_so_va_hen_tra_ket_qua;thuong_di_kem_thoi_han</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>PRED_TRAO_GIAY_TIEP_NHAN_HO_SO_VA_HEN_TRA_KET_QUA_CHO_NGU</t>
+          <t>PRED_HO_SO_BAO_GOM</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>cấp tỉnh trao giấy tiếp nhận hồ sơ và hẹn trả kết quả cho người nộp hồ sơ.</t>
+          <t>hồ sơ bao gồm</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>cấp tỉnh trao giấy tiếp nhận hồ sơ và hẹn trả kết quả cho người nộp hồ sơ. | cấp tỉnh trao giấy tiếp nhận hồ sơ và hẹn trả kết quả cho người nộp hồ sơ. với cơ quan đăng ký kinh doanh cấp tỉnh</t>
+          <t>hồ sơ bao gồm | hồ sơ bao gồm với cơ quan đăng ký kinh doanh cấp tỉnh</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -4515,7 +4523,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>trao_giay_tiep_nhan_ho_so_va_hen_tra_ket_qua_cho_nguoi_nop_ho_so</t>
+          <t>ho_so_bao_gom</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -4525,12 +4533,12 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>cơ quan đăng ký kinh doanh</t>
+          <t>công ty</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>hồ sơ đăng ký doanh nghiệp</t>
+          <t>nội dung đăng ký doanh nghiệp</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -4545,7 +4553,7 @@
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>khong</t>
+          <t>co</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
@@ -4560,49 +4568,49 @@
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>map_khi_thay_cum_trao_giay_tiep_nhan_ho_so_va_hen_tra_ket_qua_cho_nguoi_nop_ho_so</t>
+          <t>map_khi_thay_cum_ho_so_bao_gom;thuong_di_kem_thanh_phan_ho_so</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>PRED_DUNG_THUC_HIEN_THU_TUC_DANG_KY_DOANH_NGHIEP</t>
+          <t>PRED_CAC_GIAY_TO_SAU_DAY</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>dừng thực hiện thủ tục đăng ký doanh nghiệp</t>
+          <t>các giấy tờ sau đây</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>dừng thực hiện thủ tục đăng ký doanh nghiệp | dừng thực hiện thủ tục đăng ký doanh nghiệp với cơ quan đăng ký kinh doanh cấp tỉnh</t>
+          <t>các giấy tờ sau đây | các giấy tờ sau đây với cơ quan đăng ký kinh doanh cấp tỉnh</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>dang_ky</t>
+          <t>nop_ho_so</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>dung_thuc_hien_thu_tuc_dang_ky_doanh_nghiep</t>
+          <t>cac_giay_to_sau_day</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>dang_ky</t>
+          <t>nop_ho_so</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>người thành lập doanh nghiệp</t>
+          <t>công ty</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>hồ sơ đăng ký doanh nghiệp</t>
+          <t>nội dung đăng ký doanh nghiệp</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -4612,12 +4620,12 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>co</t>
+          <t>khong</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>khong</t>
+          <t>co</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
@@ -4632,24 +4640,24 @@
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>map_khi_thay_cum_dung_thuc_hien_thu_tuc_dang_ky_doanh_nghiep;uu_tien_cho_hanh_vi_dang_ky_noi_dung_phap_ly;thuong_di_kem_thoi_han</t>
+          <t>map_khi_noi_dung_la_thanh_phan_ho_so_hoac_giay_to_kem_theo</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>PRED_TRAO_GIAY_TIEP_NHAN_HO_SO_VA_HEN_TRA_KET_QUA</t>
+          <t>PRED_GUI_GIAY_DE_NGHI_DANG_KY_THAY_DOI_VON_DAU_TU_DEN_CO_</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>cấp tỉnh trao giấy tiếp nhận hồ sơ và hẹn trả kết quả</t>
+          <t>gửi giấy đề nghị đăng ký thay đổi vốn đầu tư đến Cơ quan</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>cấp tỉnh trao giấy tiếp nhận hồ sơ và hẹn trả kết quả | cấp tỉnh trao giấy tiếp nhận hồ sơ và hẹn trả kết quả với cơ quan đăng ký kinh doanh cấp tỉnh</t>
+          <t>gửi giấy đề nghị đăng ký thay đổi vốn đầu tư đến Cơ quan | gửi giấy đề nghị đăng ký thay đổi vốn đầu tư đến Cơ quan với cơ quan đăng ký kinh doanh cấp tỉnh</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -4659,7 +4667,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>trao_giay_tiep_nhan_ho_so_va_hen_tra_ket_qua</t>
+          <t>gui_giay_de_nghi_dang_ky_thay_doi_von_dau_tu_den_co_quan</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -4669,12 +4677,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>cơ quan đăng ký kinh doanh</t>
+          <t>doanh nghiệp</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Giấy chứng nhận đăng ký doanh nghiệp</t>
+          <t>giấy đề nghị</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -4684,7 +4692,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>co</t>
+          <t>khong</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4704,44 +4712,44 @@
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>map_khi_thay_cum_trao_giay_tiep_nhan_ho_so_va_hen_tra_ket_qua;thuong_di_kem_thoi_han</t>
+          <t>map_khi_thay_cum_gui_giay_de_nghi_dang_ky_thay_doi_von_dau_tu_den_co_quan</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>PRED_HO_SO_BAO_GOM</t>
+          <t>PRED_TRA_LE_PHI_DANG_KY_DOANH_NGHIEP_VA_PHI_CONG_BO_NOI_D</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>hồ sơ bao gồm</t>
+          <t>trả lệ phí đăng ký doanh nghiệp và phí công bố nội dung đăng ký doanh nghiệp trong</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>hồ sơ bao gồm | hồ sơ bao gồm với cơ quan đăng ký kinh doanh cấp tỉnh</t>
+          <t>trả lệ phí đăng ký doanh nghiệp và phí công bố nội dung đăng ký doanh nghiệp trong</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>nop_ho_so</t>
+          <t>cong_bo</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>ho_so_bao_gom</t>
+          <t>tra_le_phi_dang_ky_doanh_nghiep_va_phi_cong_bo_noi_dung_dang_ky_doanh_nghiep_trong</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>nop_ho_so</t>
+          <t>cong_bo</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>công ty</t>
+          <t>doanh nghiệp</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -4749,11 +4757,7 @@
           <t>nội dung đăng ký doanh nghiệp</t>
         </is>
       </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>cơ quan đăng ký kinh doanh cấp tỉnh</t>
-        </is>
-      </c>
+      <c r="I63" t="inlineStr"/>
       <c r="J63" t="inlineStr">
         <is>
           <t>khong</t>
@@ -4761,7 +4765,7 @@
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>co</t>
+          <t>khong</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
@@ -4776,24 +4780,24 @@
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>map_khi_thay_cum_ho_so_bao_gom;thuong_di_kem_thanh_phan_ho_so</t>
+          <t>map_khi_thay_cum_tra_le_phi_dang_ky_doanh_nghiep_va_phi_cong_bo_noi_dung_dang_ky_doanh_nghiep_trong</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>PRED_CAC_GIAY_TO_SAU_DAY</t>
+          <t>PRED_KEM_THEO_VAN_BAN_GIAI_TRINH_CUA_DOANH_NGHIEP_VE_LY_D</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>các giấy tờ sau đây</t>
+          <t>kèm theo văn bản giải trình của doanh nghiệp về lý do đăng ký thay đổi và được Cơ quan đăng ký kinh doanh cấp tỉnh chấp thuận</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>các giấy tờ sau đây | các giấy tờ sau đây với cơ quan đăng ký kinh doanh cấp tỉnh</t>
+          <t>kèm theo văn bản giải trình của doanh nghiệp về lý do đăng ký thay đổi và được Cơ quan đăng ký kinh doanh cấp tỉnh chấp thuận | kèm theo văn bản giải trình của doanh nghiệp về lý do đăng ký thay đổi và được Cơ quan đăng ký kinh doanh cấp tỉnh chấp thuận với cơ quan đăng ký kinh doanh cấp tỉnh</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -4803,7 +4807,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>cac_giay_to_sau_day</t>
+          <t>kem_theo_van_ban_giai_trinh_cua_doanh_nghiep_ve_ly_do_dang_ky_thay_doi_va_duoc_co_quan_dang_ky_kinh_doanh_cap_tinh_chap_thuan</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -4813,7 +4817,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>công ty</t>
+          <t>doanh nghiệp</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -4855,42 +4859,38 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>PRED_GUI_GIAY_DE_NGHI_DANG_KY_THAY_DOI_VON_DAU_TU_DEN_CO_</t>
+          <t>PRED_THUC_HIEN_THU_TUC_CHAM_DUT_HOAT_DONG_CHI_NHANH</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>gửi giấy đề nghị đăng ký thay đổi vốn đầu tư đến Cơ quan</t>
+          <t>thực hiện thủ tục chấm dứt hoạt động chi nhánh, văn phòng đại diện, địa điểm kinh doanh của doanh nghiệp tại Cơ quan</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>gửi giấy đề nghị đăng ký thay đổi vốn đầu tư đến Cơ quan | gửi giấy đề nghị đăng ký thay đổi vốn đầu tư đến Cơ quan với cơ quan đăng ký kinh doanh cấp tỉnh</t>
+          <t>thực hiện thủ tục chấm dứt hoạt động chi nhánh, văn phòng đại diện, địa điểm kinh doanh của doanh nghiệp tại Cơ quan | thực hiện thủ tục chấm dứt hoạt động chi nhánh, văn phòng đại diện, địa điểm kinh doanh của doanh nghiệp tại Cơ quan với cơ quan đăng ký kinh doanh cấp tỉnh</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>nop_ho_so</t>
+          <t>khac</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>gui_giay_de_nghi_dang_ky_thay_doi_von_dau_tu_den_co_quan</t>
+          <t>thuc_hien_thu_tuc_cham_dut_hoat_dong_chi_nhanh</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>nop_ho_so</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>doanh nghiệp</t>
-        </is>
-      </c>
+          <t>chi_nhanh_van_phong_dai_dien</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
-          <t>giấy đề nghị</t>
+          <t>thực hiện</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -4920,52 +4920,52 @@
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>map_khi_thay_cum_gui_giay_de_nghi_dang_ky_thay_doi_von_dau_tu_den_co_quan</t>
+          <t>map_khi_thay_cum_thuc_hien_thu_tuc_cham_dut_hoat_dong_chi_nhanh</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>PRED_TRA_LE_PHI_DANG_KY_DOANH_NGHIEP_VA_PHI_CONG_BO_NOI_D</t>
+          <t>PRED_THUC_HIEN_THU_TUC_CHAM_DUT_HOAT_DONG_CUA_TAT_CA_DIA_</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>trả lệ phí đăng ký doanh nghiệp và phí công bố nội dung đăng ký doanh nghiệp trong</t>
+          <t>thực hiện thủ tục chấm dứt hoạt động của tất cả địa điểm kinh doanh trực thuộc chi nhánh tại Cơ quan</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>trả lệ phí đăng ký doanh nghiệp và phí công bố nội dung đăng ký doanh nghiệp trong</t>
+          <t>thực hiện thủ tục chấm dứt hoạt động của tất cả địa điểm kinh doanh trực thuộc chi nhánh tại Cơ quan | thực hiện thủ tục chấm dứt hoạt động của tất cả địa điểm kinh doanh trực thuộc chi nhánh tại Cơ quan với cơ quan đăng ký kinh doanh cấp tỉnh</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>cong_bo</t>
+          <t>khac</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>tra_le_phi_dang_ky_doanh_nghiep_va_phi_cong_bo_noi_dung_dang_ky_doanh_nghiep_trong</t>
+          <t>thuc_hien_thu_tuc_cham_dut_hoat_dong_cua_tat_ca_dia_diem_kinh_doanh_truc_thuoc_chi_nhanh_tai_co_quan</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>cong_bo</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>doanh nghiệp</t>
-        </is>
-      </c>
+          <t>chi_nhanh_van_phong_dai_dien</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
         <is>
-          <t>nội dung đăng ký doanh nghiệp</t>
-        </is>
-      </c>
-      <c r="I66" t="inlineStr"/>
+          <t>thực hiện</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>cơ quan đăng ký kinh doanh cấp tỉnh</t>
+        </is>
+      </c>
       <c r="J66" t="inlineStr">
         <is>
           <t>khong</t>
@@ -4988,49 +4988,49 @@
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t>map_khi_thay_cum_tra_le_phi_dang_ky_doanh_nghiep_va_phi_cong_bo_noi_dung_dang_ky_doanh_nghiep_trong</t>
+          <t>map_khi_thay_cum_thuc_hien_thu_tuc_cham_dut_hoat_dong_cua_tat_ca_dia_diem_kinh_doanh_truc_thuoc_chi_nhanh_tai_co_quan</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>PRED_KEM_THEO_VAN_BAN_GIAI_TRINH_CUA_DOANH_NGHIEP_VE_LY_D</t>
+          <t>PRED_THONG_BAO_CHO_CO_QUAN_QUAN_LY_THUE</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>kèm theo văn bản giải trình của doanh nghiệp về lý do đăng ký thay đổi và được Cơ quan đăng ký kinh doanh cấp tỉnh chấp thuận</t>
+          <t>cấp tỉnh thông báo cho Cơ quan quản lý thuế</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>kèm theo văn bản giải trình của doanh nghiệp về lý do đăng ký thay đổi và được Cơ quan đăng ký kinh doanh cấp tỉnh chấp thuận | kèm theo văn bản giải trình của doanh nghiệp về lý do đăng ký thay đổi và được Cơ quan đăng ký kinh doanh cấp tỉnh chấp thuận với cơ quan đăng ký kinh doanh cấp tỉnh</t>
+          <t>cấp tỉnh thông báo cho Cơ quan quản lý thuế | cấp tỉnh thông báo cho Cơ quan quản lý thuế với cơ quan đăng ký kinh doanh cấp tỉnh</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>nop_ho_so</t>
+          <t>thong_bao</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>kem_theo_van_ban_giai_trinh_cua_doanh_nghiep_ve_ly_do_dang_ky_thay_doi_va_duoc_co_quan_dang_ky_kinh_doanh_cap_tinh_chap_thuan</t>
+          <t>thong_bao_cho_co_quan_quan_ly_thue</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>nop_ho_so</t>
+          <t>thong_bao</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>doanh nghiệp</t>
+          <t>cơ quan đăng ký kinh doanh</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>nội dung đăng ký doanh nghiệp</t>
+          <t>Giấy chứng nhận đăng ký doanh nghiệp</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -5040,12 +5040,12 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>khong</t>
+          <t>co</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>co</t>
+          <t>khong</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
@@ -5060,45 +5060,49 @@
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t>map_khi_noi_dung_la_thanh_phan_ho_so_hoac_giay_to_kem_theo</t>
+          <t>map_khi_thay_cum_thong_bao_cho_co_quan_quan_ly_thue;khong_dong_nhat_voi_cong_bo;thuong_di_kem_thoi_han</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>PRED_THUC_HIEN_THU_TUC_CHAM_DUT_HOAT_DONG_CHI_NHANH</t>
+          <t>PRED_HUY_BO_QUYET_DINH_THU_HOI</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>thực hiện thủ tục chấm dứt hoạt động chi nhánh, văn phòng đại diện, địa điểm kinh doanh của doanh nghiệp tại Cơ quan</t>
+          <t>cấp tỉnh ra quyết định hủy bỏ quyết định thu hồi và khôi phục Giấy chứng nhận đăng ký doanh nghiệp</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>thực hiện thủ tục chấm dứt hoạt động chi nhánh, văn phòng đại diện, địa điểm kinh doanh của doanh nghiệp tại Cơ quan | thực hiện thủ tục chấm dứt hoạt động chi nhánh, văn phòng đại diện, địa điểm kinh doanh của doanh nghiệp tại Cơ quan với cơ quan đăng ký kinh doanh cấp tỉnh</t>
+          <t>cấp tỉnh ra quyết định hủy bỏ quyết định thu hồi và khôi phục Giấy chứng nhận đăng ký doanh nghiệp | cấp tỉnh ra quyết định hủy bỏ quyết định thu hồi và khôi phục Giấy chứng nhận đăng ký doanh nghiệp với cơ quan đăng ký kinh doanh cấp tỉnh</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>khac</t>
+          <t>thu_hoi</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>thuc_hien_thu_tuc_cham_dut_hoat_dong_chi_nhanh</t>
+          <t>huy_bo_quyet_dinh_thu_hoi</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>chi_nhanh_van_phong_dai_dien</t>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr"/>
+          <t>thu_hoi</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>cơ quan đăng ký kinh doanh</t>
+        </is>
+      </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>thực hiện</t>
+          <t>Giấy chứng nhận đăng ký doanh nghiệp</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -5108,7 +5112,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>khong</t>
+          <t>co</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -5128,50 +5132,54 @@
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t>map_khi_thay_cum_thuc_hien_thu_tuc_cham_dut_hoat_dong_chi_nhanh</t>
+          <t>map_khi_thay_cum_huy_bo_quyet_dinh_thu_hoi;thuong_di_kem_thoi_han</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>PRED_THUC_HIEN_THU_TUC_CHAM_DUT_HOAT_DONG_CUA_TAT_CA_DIA_</t>
+          <t>PRED_CO_QUAN_DANG_KY_KINH_DOANH</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>thực hiện thủ tục chấm dứt hoạt động của tất cả địa điểm kinh doanh trực thuộc chi nhánh tại Cơ quan</t>
+          <t>Cơ quan đăng ký kinh doanh</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>thực hiện thủ tục chấm dứt hoạt động của tất cả địa điểm kinh doanh trực thuộc chi nhánh tại Cơ quan | thực hiện thủ tục chấm dứt hoạt động của tất cả địa điểm kinh doanh trực thuộc chi nhánh tại Cơ quan với cơ quan đăng ký kinh doanh cấp tỉnh</t>
+          <t>Cơ quan đăng ký kinh doanh | Cơ quan đăng ký kinh doanh với cơ quan đăng ký kinh doanh</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>khac</t>
+          <t>dang_ky</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>thuc_hien_thu_tuc_cham_dut_hoat_dong_cua_tat_ca_dia_diem_kinh_doanh_truc_thuoc_chi_nhanh_tai_co_quan</t>
+          <t>co_quan_dang_ky_kinh_doanh</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>chi_nhanh_van_phong_dai_dien</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr"/>
+          <t>dang_ky</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>cơ quan đăng ký kinh doanh</t>
+        </is>
+      </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>thực hiện</t>
+          <t>cấp xã và các cơ quan khác gây phiền hà đối với tổ chức</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>cơ quan đăng ký kinh doanh cấp tỉnh</t>
+          <t>cơ quan đăng ký kinh doanh</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -5196,59 +5204,59 @@
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t>map_khi_thay_cum_thuc_hien_thu_tuc_cham_dut_hoat_dong_cua_tat_ca_dia_diem_kinh_doanh_truc_thuoc_chi_nhanh_tai_co_quan</t>
+          <t>map_khi_thay_cum_co_quan_dang_ky_kinh_doanh;uu_tien_cho_hanh_vi_dang_ky_noi_dung_phap_ly</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>PRED_DANG_KY_DOANH_NGHIEP</t>
+          <t>PRED_XA_TIEP_NHAN_HO_SO_DANG_KY_HO_KINH_DOANH_VAO_HE_THON</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>đăng ký kinh doanh cấp tỉnh ra thông báo về việc vi phạm của doanh nghiệp và quyết định thu hồi Giấy chứng nhận đăng ký doanh nghiệp</t>
+          <t>xã tiếp nhận hồ sơ đăng ký hộ kinh doanh vào Hệ thống thông tin về đăng ký hộ kinh doanh</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>đăng ký kinh doanh cấp tỉnh ra thông báo về việc vi phạm của doanh nghiệp và quyết định thu hồi Giấy chứng nhận đăng ký doanh nghiệp | đăng ký kinh doanh cấp tỉnh ra thông báo về việc vi phạm của doanh nghiệp và quyết định thu hồi Giấy chứng nhận đăng ký doanh nghiệp với cơ quan đăng ký kinh doanh cấp tỉnh</t>
+          <t>xã tiếp nhận hồ sơ đăng ký hộ kinh doanh vào Hệ thống thông tin về đăng ký hộ kinh doanh | xã tiếp nhận hồ sơ đăng ký hộ kinh doanh vào Hệ thống thông tin về đăng ký hộ kinh doanh với cơ quan đăng ký kinh doanh</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>dang_ky</t>
+          <t>nop_ho_so</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>dang_ky_doanh_nghiep</t>
+          <t>xa_tiep_nhan_ho_so_dang_ky_ho_kinh_doanh_vao_he_thong_thong_tin_ve_dang_ky_ho_kinh_doanh</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>thong_bao</t>
+          <t>nop_ho_so</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>doanh nghiệp</t>
+          <t>cơ quan đăng ký kinh doanh</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>thời hạn 03 ngày làm việc kể từ ngày nhận được giấy tờ quy định tại khoản 2 Điều 68 Nghị định này</t>
+          <t>hồ sơ đáp ứng các điều kiện sau đây:</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>cơ quan đăng ký kinh doanh cấp tỉnh</t>
+          <t>cơ quan đăng ký kinh doanh</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>co</t>
+          <t>khong</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -5263,368 +5271,12 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>co</t>
+          <t>khong</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
         <is>
-          <t>map_khi_thay_cum_dang_ky_doanh_nghiep;khong_dong_nhat_voi_cong_bo;thuong_di_kem_thoi_han</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>PRED_THONG_BAO_CHO_CO_QUAN_QUAN_LY_THUE</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>cấp tỉnh thông báo cho Cơ quan quản lý thuế</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>cấp tỉnh thông báo cho Cơ quan quản lý thuế | cấp tỉnh thông báo cho Cơ quan quản lý thuế với cơ quan đăng ký kinh doanh cấp tỉnh</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>thong_bao</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>thong_bao_cho_co_quan_quan_ly_thue</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>thong_bao</t>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>cơ quan đăng ký kinh doanh</t>
-        </is>
-      </c>
-      <c r="H71" t="inlineStr">
-        <is>
-          <t>Giấy chứng nhận đăng ký doanh nghiệp</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>cơ quan đăng ký kinh doanh cấp tỉnh</t>
-        </is>
-      </c>
-      <c r="J71" t="inlineStr">
-        <is>
-          <t>co</t>
-        </is>
-      </c>
-      <c r="K71" t="inlineStr">
-        <is>
-          <t>khong</t>
-        </is>
-      </c>
-      <c r="L71" t="inlineStr">
-        <is>
-          <t>khong</t>
-        </is>
-      </c>
-      <c r="M71" t="inlineStr">
-        <is>
-          <t>khong</t>
-        </is>
-      </c>
-      <c r="N71" t="inlineStr">
-        <is>
-          <t>map_khi_thay_cum_thong_bao_cho_co_quan_quan_ly_thue;khong_dong_nhat_voi_cong_bo;thuong_di_kem_thoi_han</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>PRED_HUY_BO_QUYET_DINH_THU_HOI</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>cấp tỉnh ra quyết định hủy bỏ quyết định thu hồi và khôi phục Giấy chứng nhận đăng ký doanh nghiệp</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>cấp tỉnh ra quyết định hủy bỏ quyết định thu hồi và khôi phục Giấy chứng nhận đăng ký doanh nghiệp | cấp tỉnh ra quyết định hủy bỏ quyết định thu hồi và khôi phục Giấy chứng nhận đăng ký doanh nghiệp với cơ quan đăng ký kinh doanh cấp tỉnh</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>thu_hoi</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>huy_bo_quyet_dinh_thu_hoi</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>thu_hoi</t>
-        </is>
-      </c>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>cơ quan đăng ký kinh doanh</t>
-        </is>
-      </c>
-      <c r="H72" t="inlineStr">
-        <is>
-          <t>Giấy chứng nhận đăng ký doanh nghiệp</t>
-        </is>
-      </c>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t>cơ quan đăng ký kinh doanh cấp tỉnh</t>
-        </is>
-      </c>
-      <c r="J72" t="inlineStr">
-        <is>
-          <t>co</t>
-        </is>
-      </c>
-      <c r="K72" t="inlineStr">
-        <is>
-          <t>khong</t>
-        </is>
-      </c>
-      <c r="L72" t="inlineStr">
-        <is>
-          <t>khong</t>
-        </is>
-      </c>
-      <c r="M72" t="inlineStr">
-        <is>
-          <t>khong</t>
-        </is>
-      </c>
-      <c r="N72" t="inlineStr">
-        <is>
-          <t>map_khi_thay_cum_huy_bo_quyet_dinh_thu_hoi;thuong_di_kem_thoi_han</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>PRED_CO_QUAN_DANG_KY_KINH_DOANH</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>Cơ quan đăng ký kinh doanh</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>Cơ quan đăng ký kinh doanh | Cơ quan đăng ký kinh doanh với cơ quan đăng ký kinh doanh</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>dang_ky</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>co_quan_dang_ky_kinh_doanh</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>dang_ky</t>
-        </is>
-      </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>cơ quan đăng ký kinh doanh</t>
-        </is>
-      </c>
-      <c r="H73" t="inlineStr">
-        <is>
-          <t>cấp xã và các cơ quan khác gây phiền hà đối với tổ chức</t>
-        </is>
-      </c>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t>cơ quan đăng ký kinh doanh</t>
-        </is>
-      </c>
-      <c r="J73" t="inlineStr">
-        <is>
-          <t>khong</t>
-        </is>
-      </c>
-      <c r="K73" t="inlineStr">
-        <is>
-          <t>khong</t>
-        </is>
-      </c>
-      <c r="L73" t="inlineStr">
-        <is>
-          <t>khong</t>
-        </is>
-      </c>
-      <c r="M73" t="inlineStr">
-        <is>
-          <t>khong</t>
-        </is>
-      </c>
-      <c r="N73" t="inlineStr">
-        <is>
-          <t>map_khi_thay_cum_co_quan_dang_ky_kinh_doanh;uu_tien_cho_hanh_vi_dang_ky_noi_dung_phap_ly</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>PRED_XA_TIEP_NHAN_HO_SO_DANG_KY_HO_KINH_DOANH_VAO_HE_THON</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>xã tiếp nhận hồ sơ đăng ký hộ kinh doanh vào Hệ thống thông tin về đăng ký hộ kinh doanh</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>xã tiếp nhận hồ sơ đăng ký hộ kinh doanh vào Hệ thống thông tin về đăng ký hộ kinh doanh | xã tiếp nhận hồ sơ đăng ký hộ kinh doanh vào Hệ thống thông tin về đăng ký hộ kinh doanh với cơ quan đăng ký kinh doanh</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>nop_ho_so</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>xa_tiep_nhan_ho_so_dang_ky_ho_kinh_doanh_vao_he_thong_thong_tin_ve_dang_ky_ho_kinh_doanh</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>nop_ho_so</t>
-        </is>
-      </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>cơ quan đăng ký kinh doanh</t>
-        </is>
-      </c>
-      <c r="H74" t="inlineStr">
-        <is>
-          <t>hồ sơ đáp ứng các điều kiện sau đây:</t>
-        </is>
-      </c>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>cơ quan đăng ký kinh doanh</t>
-        </is>
-      </c>
-      <c r="J74" t="inlineStr">
-        <is>
-          <t>khong</t>
-        </is>
-      </c>
-      <c r="K74" t="inlineStr">
-        <is>
-          <t>khong</t>
-        </is>
-      </c>
-      <c r="L74" t="inlineStr">
-        <is>
-          <t>khong</t>
-        </is>
-      </c>
-      <c r="M74" t="inlineStr">
-        <is>
-          <t>khong</t>
-        </is>
-      </c>
-      <c r="N74" t="inlineStr">
-        <is>
           <t>map_khi_thay_cum_xa_tiep_nhan_ho_so_dang_ky_ho_kinh_doanh_vao_he_thong_thong_tin_ve_dang_ky_ho_kinh_doanh</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>PRED_CAP_CO_SU_DUNG_THONG_TIN_TU_CHUNG_MINH_NHAN_DAN</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>cấp có sử dụng thông tin từ chứng minh nhân dân</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>cấp có sử dụng thông tin từ chứng minh nhân dân | cấp có sử dụng thông tin từ chứng minh nhân dân với cơ quan đăng ký kinh doanh</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>khac</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>cap_co_su_dung_thong_tin_tu_chung_minh_nhan_dan</t>
-        </is>
-      </c>
-      <c r="F75" t="inlineStr">
-        <is>
-          <t>hanh_dong_co_quan</t>
-        </is>
-      </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>cơ quan đăng ký kinh doanh</t>
-        </is>
-      </c>
-      <c r="H75" t="inlineStr"/>
-      <c r="I75" t="inlineStr">
-        <is>
-          <t>cơ quan đăng ký kinh doanh</t>
-        </is>
-      </c>
-      <c r="J75" t="inlineStr">
-        <is>
-          <t>khong</t>
-        </is>
-      </c>
-      <c r="K75" t="inlineStr">
-        <is>
-          <t>khong</t>
-        </is>
-      </c>
-      <c r="L75" t="inlineStr">
-        <is>
-          <t>khong</t>
-        </is>
-      </c>
-      <c r="M75" t="inlineStr">
-        <is>
-          <t>khong</t>
-        </is>
-      </c>
-      <c r="N75" t="inlineStr">
-        <is>
-          <t>map_khi_thay_cum_cap_co_su_dung_thong_tin_tu_chung_minh_nhan_dan</t>
         </is>
       </c>
     </row>

</xml_diff>